<commit_message>
SBMD-13 test: ornek Excel gercek il/ilce kodlariyla yeniden uretildi
Ilce kodlari uydurma degil, Temmuz 2026 uretim ekstresindeki gercek ciftler:
34/0, 35/0, 6/0 (buyuksehir) ve 2/1105, 3/1108, 3/1306 (ilce bazli).
Boylece SBM'den RISK-HAVUZU-00009 (ilce bulunamadi) beklenmez.
Hatali satir dosyasi da ayni gercek kodlarla yeniden uretildi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pentest-ornek-beyanname.xlsx
+++ b/pentest-ornek-beyanname.xlsx
@@ -770,10 +770,10 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>2201</v>
+        <v>1105</v>
       </c>
       <c r="D8" t="n">
         <v>2320</v>
@@ -813,10 +813,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>2201</v>
+        <v>1105</v>
       </c>
       <c r="D9" t="n">
         <v>2320</v>
@@ -856,10 +856,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>47</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>4703</v>
+        <v>1108</v>
       </c>
       <c r="D10" t="n">
         <v>2320</v>
@@ -899,10 +899,10 @@
         <v>8</v>
       </c>
       <c r="B11" t="n">
-        <v>47</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>4703</v>
+        <v>1108</v>
       </c>
       <c r="D11" t="n">
         <v>2320</v>
@@ -942,10 +942,10 @@
         <v>8</v>
       </c>
       <c r="B12" t="n">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>6801</v>
+        <v>1306</v>
       </c>
       <c r="D12" t="n">
         <v>2320</v>
@@ -985,10 +985,10 @@
         <v>8</v>
       </c>
       <c r="B13" t="n">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>6801</v>
+        <v>1306</v>
       </c>
       <c r="D13" t="n">
         <v>2320</v>

</xml_diff>